<commit_message>
fix(wilcock): compute tau_ri as the hydrologist does
- scale the Shields number by (di/D50)^b and convert with each fraction's own di (D50), so tau_ri reproduces the sample file to its rounding
- regenerate the B3.2 workbook (new tau_ri* column) and CSVs, rewrite the tau_ri tests around the sample file, update the before and after table
- B3.2, D36, D50, AL-02 and OI-04; the form departs from W&C Eqs. 3 and 5 and needs hydrologist confirmation
</commit_message>
<xml_diff>
--- a/tests/verification/bedload_verification.xlsx
+++ b/tests/verification/bedload_verification.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -568,21 +568,10 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>tau_rm = tau_rm* (s-1) rho_w g D50 (Pa)</t>
+          <t>Mass factor rho_s / 1000 (t/m3)</t>
         </is>
       </c>
       <c r="B14">
-        <f>B13*(B12-1)*B3*B2*B8</f>
-        <v/>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>Mass factor rho_s / 1000 (t/m3)</t>
-        </is>
-      </c>
-      <c r="B15">
         <f>B4/1000</f>
         <v/>
       </c>
@@ -810,14 +799,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:H8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="34" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="38" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -843,10 +833,15 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>tau_ri = tau_rm (di/D50)^b_i (Pa)</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
+          <t>tau_ri* = tau_rm* (di/D50)^b_i</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>tau_ri = tau_ri* (s-1) rho_w g di (Pa)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
         <is>
           <t>Rows without Fi only check tau_ri.</t>
         </is>
@@ -868,7 +863,11 @@
         <v/>
       </c>
       <c r="E2">
-        <f>Constants!$B$14*C2^D2</f>
+        <f>Constants!$B$13*C2^D2</f>
+        <v/>
+      </c>
+      <c r="F2">
+        <f>E2*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A2</f>
         <v/>
       </c>
     </row>
@@ -888,7 +887,11 @@
         <v/>
       </c>
       <c r="E3">
-        <f>Constants!$B$14*C3^D3</f>
+        <f>Constants!$B$13*C3^D3</f>
+        <v/>
+      </c>
+      <c r="F3">
+        <f>E3*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A3</f>
         <v/>
       </c>
     </row>
@@ -908,7 +911,11 @@
         <v/>
       </c>
       <c r="E4">
-        <f>Constants!$B$14*C4^D4</f>
+        <f>Constants!$B$13*C4^D4</f>
+        <v/>
+      </c>
+      <c r="F4">
+        <f>E4*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A4</f>
         <v/>
       </c>
     </row>
@@ -928,7 +935,11 @@
         <v/>
       </c>
       <c r="E5">
-        <f>Constants!$B$14*C5^D5</f>
+        <f>Constants!$B$13*C5^D5</f>
+        <v/>
+      </c>
+      <c r="F5">
+        <f>E5*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A5</f>
         <v/>
       </c>
     </row>
@@ -948,7 +959,11 @@
         <v/>
       </c>
       <c r="E6">
-        <f>Constants!$B$14*C6^D6</f>
+        <f>Constants!$B$13*C6^D6</f>
+        <v/>
+      </c>
+      <c r="F6">
+        <f>E6*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A6</f>
         <v/>
       </c>
     </row>
@@ -965,7 +980,11 @@
         <v/>
       </c>
       <c r="E7">
-        <f>Constants!$B$14*C7^D7</f>
+        <f>Constants!$B$13*C7^D7</f>
+        <v/>
+      </c>
+      <c r="F7">
+        <f>E7*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A7</f>
         <v/>
       </c>
     </row>
@@ -982,7 +1001,11 @@
         <v/>
       </c>
       <c r="E8">
-        <f>Constants!$B$14*C8^D8</f>
+        <f>Constants!$B$13*C8^D8</f>
+        <v/>
+      </c>
+      <c r="F8">
+        <f>E8*(Constants!$B$12-1)*Constants!$B$3*Constants!$B$2*A8</f>
         <v/>
       </c>
     </row>
@@ -1101,7 +1124,7 @@
         <v/>
       </c>
       <c r="G2">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H2">
@@ -1149,7 +1172,7 @@
         <v/>
       </c>
       <c r="G3">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H3">
@@ -1197,7 +1220,7 @@
         <v/>
       </c>
       <c r="G4">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H4">
@@ -1245,7 +1268,7 @@
         <v/>
       </c>
       <c r="G5">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H5">
@@ -1293,7 +1316,7 @@
         <v/>
       </c>
       <c r="G6">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H6">
@@ -1341,7 +1364,7 @@
         <v/>
       </c>
       <c r="G7">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H7">
@@ -1389,7 +1412,7 @@
         <v/>
       </c>
       <c r="G8">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H8">
@@ -1437,7 +1460,7 @@
         <v/>
       </c>
       <c r="G9">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H9">
@@ -1485,7 +1508,7 @@
         <v/>
       </c>
       <c r="G10">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H10">
@@ -1526,7 +1549,7 @@
         <v/>
       </c>
       <c r="G11">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H11">
@@ -1567,7 +1590,7 @@
         <v/>
       </c>
       <c r="G12">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H12">
@@ -1608,7 +1631,7 @@
         <v/>
       </c>
       <c r="G13">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H13">
@@ -1649,7 +1672,7 @@
         <v/>
       </c>
       <c r="G14">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H14">
@@ -1690,7 +1713,7 @@
         <v/>
       </c>
       <c r="G15">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H15">
@@ -1731,7 +1754,7 @@
         <v/>
       </c>
       <c r="G16">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H16">
@@ -1772,7 +1795,7 @@
         <v/>
       </c>
       <c r="G17">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H17">
@@ -1813,7 +1836,7 @@
         <v/>
       </c>
       <c r="G18">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H18">
@@ -1854,7 +1877,7 @@
         <v/>
       </c>
       <c r="G19">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H19">
@@ -1895,7 +1918,7 @@
         <v/>
       </c>
       <c r="G20">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H20">
@@ -1936,7 +1959,7 @@
         <v/>
       </c>
       <c r="G21">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H21">
@@ -1977,7 +2000,7 @@
         <v/>
       </c>
       <c r="G22">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H22">
@@ -2018,7 +2041,7 @@
         <v/>
       </c>
       <c r="G23">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H23">
@@ -2059,7 +2082,7 @@
         <v/>
       </c>
       <c r="G24">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H24">
@@ -2100,7 +2123,7 @@
         <v/>
       </c>
       <c r="G25">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H25">
@@ -2141,7 +2164,7 @@
         <v/>
       </c>
       <c r="G26">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H26">
@@ -2182,7 +2205,7 @@
         <v/>
       </c>
       <c r="G27">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H27">
@@ -2223,7 +2246,7 @@
         <v/>
       </c>
       <c r="G28">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H28">
@@ -2264,7 +2287,7 @@
         <v/>
       </c>
       <c r="G29">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H29">
@@ -2305,7 +2328,7 @@
         <v/>
       </c>
       <c r="G30">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H30">
@@ -2346,7 +2369,7 @@
         <v/>
       </c>
       <c r="G31">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H31">
@@ -2387,7 +2410,7 @@
         <v/>
       </c>
       <c r="G32">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H32">
@@ -2428,7 +2451,7 @@
         <v/>
       </c>
       <c r="G33">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H33">
@@ -2469,7 +2492,7 @@
         <v/>
       </c>
       <c r="G34">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H34">
@@ -2510,7 +2533,7 @@
         <v/>
       </c>
       <c r="G35">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H35">
@@ -2551,7 +2574,7 @@
         <v/>
       </c>
       <c r="G36">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H36">
@@ -2592,7 +2615,7 @@
         <v/>
       </c>
       <c r="G37">
-        <f>Fractions!$E$2</f>
+        <f>Fractions!$F$2</f>
         <v/>
       </c>
       <c r="H37">
@@ -2633,7 +2656,7 @@
         <v/>
       </c>
       <c r="G38">
-        <f>Fractions!$E$3</f>
+        <f>Fractions!$F$3</f>
         <v/>
       </c>
       <c r="H38">
@@ -2674,7 +2697,7 @@
         <v/>
       </c>
       <c r="G39">
-        <f>Fractions!$E$4</f>
+        <f>Fractions!$F$4</f>
         <v/>
       </c>
       <c r="H39">
@@ -2715,7 +2738,7 @@
         <v/>
       </c>
       <c r="G40">
-        <f>Fractions!$E$5</f>
+        <f>Fractions!$F$5</f>
         <v/>
       </c>
       <c r="H40">
@@ -2756,7 +2779,7 @@
         <v/>
       </c>
       <c r="G41">
-        <f>Fractions!$E$6</f>
+        <f>Fractions!$F$6</f>
         <v/>
       </c>
       <c r="H41">
@@ -2916,23 +2939,23 @@
         <v/>
       </c>
       <c r="G2">
-        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$E$2&lt;Constants!$B$10,0.002*(E2/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E2/Fractions!$E$2))^4.5))*Fractions!$B$2*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$F$2&lt;Constants!$B$10,0.002*(E2/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E2/Fractions!$F$2))^4.5))*Fractions!$B$2*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H2">
-        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$E$3&lt;Constants!$B$10,0.002*(E2/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E2/Fractions!$E$3))^4.5))*Fractions!$B$3*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$F$3&lt;Constants!$B$10,0.002*(E2/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E2/Fractions!$F$3))^4.5))*Fractions!$B$3*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I2">
-        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$E$4&lt;Constants!$B$10,0.002*(E2/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E2/Fractions!$E$4))^4.5))*Fractions!$B$4*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$F$4&lt;Constants!$B$10,0.002*(E2/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E2/Fractions!$F$4))^4.5))*Fractions!$B$4*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J2">
-        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$E$5&lt;Constants!$B$10,0.002*(E2/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E2/Fractions!$E$5))^4.5))*Fractions!$B$5*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$F$5&lt;Constants!$B$10,0.002*(E2/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E2/Fractions!$F$5))^4.5))*Fractions!$B$5*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K2">
-        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$E$6&lt;Constants!$B$10,0.002*(E2/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E2/Fractions!$E$6))^4.5))*Fractions!$B$6*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E2&lt;=0,0,IF(E2/Fractions!$F$6&lt;Constants!$B$10,0.002*(E2/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E2/Fractions!$F$6))^4.5))*Fractions!$B$6*F2^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L2">
@@ -2964,7 +2987,7 @@
         <v/>
       </c>
       <c r="T2">
-        <f>S2*Constants!$B$15</f>
+        <f>S2*Constants!$B$14</f>
         <v/>
       </c>
     </row>
@@ -2992,23 +3015,23 @@
         <v/>
       </c>
       <c r="G3">
-        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$E$2&lt;Constants!$B$10,0.002*(E3/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E3/Fractions!$E$2))^4.5))*Fractions!$B$2*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$F$2&lt;Constants!$B$10,0.002*(E3/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E3/Fractions!$F$2))^4.5))*Fractions!$B$2*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H3">
-        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$E$3&lt;Constants!$B$10,0.002*(E3/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E3/Fractions!$E$3))^4.5))*Fractions!$B$3*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$F$3&lt;Constants!$B$10,0.002*(E3/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E3/Fractions!$F$3))^4.5))*Fractions!$B$3*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I3">
-        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$E$4&lt;Constants!$B$10,0.002*(E3/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E3/Fractions!$E$4))^4.5))*Fractions!$B$4*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$F$4&lt;Constants!$B$10,0.002*(E3/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E3/Fractions!$F$4))^4.5))*Fractions!$B$4*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J3">
-        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$E$5&lt;Constants!$B$10,0.002*(E3/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E3/Fractions!$E$5))^4.5))*Fractions!$B$5*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$F$5&lt;Constants!$B$10,0.002*(E3/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E3/Fractions!$F$5))^4.5))*Fractions!$B$5*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K3">
-        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$E$6&lt;Constants!$B$10,0.002*(E3/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E3/Fractions!$E$6))^4.5))*Fractions!$B$6*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E3&lt;=0,0,IF(E3/Fractions!$F$6&lt;Constants!$B$10,0.002*(E3/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E3/Fractions!$F$6))^4.5))*Fractions!$B$6*F3^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L3">
@@ -3040,7 +3063,7 @@
         <v/>
       </c>
       <c r="T3">
-        <f>S3*Constants!$B$15</f>
+        <f>S3*Constants!$B$14</f>
         <v/>
       </c>
     </row>
@@ -3068,23 +3091,23 @@
         <v/>
       </c>
       <c r="G4">
-        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$E$2&lt;Constants!$B$10,0.002*(E4/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E4/Fractions!$E$2))^4.5))*Fractions!$B$2*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$F$2&lt;Constants!$B$10,0.002*(E4/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E4/Fractions!$F$2))^4.5))*Fractions!$B$2*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H4">
-        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$E$3&lt;Constants!$B$10,0.002*(E4/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E4/Fractions!$E$3))^4.5))*Fractions!$B$3*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$F$3&lt;Constants!$B$10,0.002*(E4/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E4/Fractions!$F$3))^4.5))*Fractions!$B$3*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I4">
-        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$E$4&lt;Constants!$B$10,0.002*(E4/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E4/Fractions!$E$4))^4.5))*Fractions!$B$4*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$F$4&lt;Constants!$B$10,0.002*(E4/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E4/Fractions!$F$4))^4.5))*Fractions!$B$4*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J4">
-        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$E$5&lt;Constants!$B$10,0.002*(E4/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E4/Fractions!$E$5))^4.5))*Fractions!$B$5*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$F$5&lt;Constants!$B$10,0.002*(E4/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E4/Fractions!$F$5))^4.5))*Fractions!$B$5*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K4">
-        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$E$6&lt;Constants!$B$10,0.002*(E4/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E4/Fractions!$E$6))^4.5))*Fractions!$B$6*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E4&lt;=0,0,IF(E4/Fractions!$F$6&lt;Constants!$B$10,0.002*(E4/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E4/Fractions!$F$6))^4.5))*Fractions!$B$6*F4^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L4">
@@ -3116,7 +3139,7 @@
         <v/>
       </c>
       <c r="T4">
-        <f>S4*Constants!$B$15</f>
+        <f>S4*Constants!$B$14</f>
         <v/>
       </c>
     </row>
@@ -3144,23 +3167,23 @@
         <v/>
       </c>
       <c r="G5">
-        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$E$2&lt;Constants!$B$10,0.002*(E5/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E5/Fractions!$E$2))^4.5))*Fractions!$B$2*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$F$2&lt;Constants!$B$10,0.002*(E5/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E5/Fractions!$F$2))^4.5))*Fractions!$B$2*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H5">
-        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$E$3&lt;Constants!$B$10,0.002*(E5/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E5/Fractions!$E$3))^4.5))*Fractions!$B$3*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$F$3&lt;Constants!$B$10,0.002*(E5/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E5/Fractions!$F$3))^4.5))*Fractions!$B$3*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I5">
-        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$E$4&lt;Constants!$B$10,0.002*(E5/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E5/Fractions!$E$4))^4.5))*Fractions!$B$4*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$F$4&lt;Constants!$B$10,0.002*(E5/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E5/Fractions!$F$4))^4.5))*Fractions!$B$4*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J5">
-        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$E$5&lt;Constants!$B$10,0.002*(E5/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E5/Fractions!$E$5))^4.5))*Fractions!$B$5*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$F$5&lt;Constants!$B$10,0.002*(E5/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E5/Fractions!$F$5))^4.5))*Fractions!$B$5*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K5">
-        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$E$6&lt;Constants!$B$10,0.002*(E5/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E5/Fractions!$E$6))^4.5))*Fractions!$B$6*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E5&lt;=0,0,IF(E5/Fractions!$F$6&lt;Constants!$B$10,0.002*(E5/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E5/Fractions!$F$6))^4.5))*Fractions!$B$6*F5^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L5">
@@ -3192,7 +3215,7 @@
         <v/>
       </c>
       <c r="T5">
-        <f>S5*Constants!$B$15</f>
+        <f>S5*Constants!$B$14</f>
         <v/>
       </c>
     </row>
@@ -3220,23 +3243,23 @@
         <v/>
       </c>
       <c r="G6">
-        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$E$2&lt;Constants!$B$10,0.002*(E6/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E6/Fractions!$E$2))^4.5))*Fractions!$B$2*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$F$2&lt;Constants!$B$10,0.002*(E6/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E6/Fractions!$F$2))^4.5))*Fractions!$B$2*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H6">
-        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$E$3&lt;Constants!$B$10,0.002*(E6/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E6/Fractions!$E$3))^4.5))*Fractions!$B$3*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$F$3&lt;Constants!$B$10,0.002*(E6/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E6/Fractions!$F$3))^4.5))*Fractions!$B$3*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I6">
-        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$E$4&lt;Constants!$B$10,0.002*(E6/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E6/Fractions!$E$4))^4.5))*Fractions!$B$4*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$F$4&lt;Constants!$B$10,0.002*(E6/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E6/Fractions!$F$4))^4.5))*Fractions!$B$4*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J6">
-        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$E$5&lt;Constants!$B$10,0.002*(E6/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E6/Fractions!$E$5))^4.5))*Fractions!$B$5*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$F$5&lt;Constants!$B$10,0.002*(E6/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E6/Fractions!$F$5))^4.5))*Fractions!$B$5*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K6">
-        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$E$6&lt;Constants!$B$10,0.002*(E6/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E6/Fractions!$E$6))^4.5))*Fractions!$B$6*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E6&lt;=0,0,IF(E6/Fractions!$F$6&lt;Constants!$B$10,0.002*(E6/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E6/Fractions!$F$6))^4.5))*Fractions!$B$6*F6^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L6">
@@ -3268,7 +3291,7 @@
         <v/>
       </c>
       <c r="T6">
-        <f>S6*Constants!$B$15</f>
+        <f>S6*Constants!$B$14</f>
         <v/>
       </c>
     </row>
@@ -3296,23 +3319,23 @@
         <v/>
       </c>
       <c r="G7">
-        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$E$2&lt;Constants!$B$10,0.002*(E7/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E7/Fractions!$E$2))^4.5))*Fractions!$B$2*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$F$2&lt;Constants!$B$10,0.002*(E7/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E7/Fractions!$F$2))^4.5))*Fractions!$B$2*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H7">
-        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$E$3&lt;Constants!$B$10,0.002*(E7/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E7/Fractions!$E$3))^4.5))*Fractions!$B$3*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$F$3&lt;Constants!$B$10,0.002*(E7/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E7/Fractions!$F$3))^4.5))*Fractions!$B$3*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I7">
-        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$E$4&lt;Constants!$B$10,0.002*(E7/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E7/Fractions!$E$4))^4.5))*Fractions!$B$4*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$F$4&lt;Constants!$B$10,0.002*(E7/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E7/Fractions!$F$4))^4.5))*Fractions!$B$4*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J7">
-        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$E$5&lt;Constants!$B$10,0.002*(E7/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E7/Fractions!$E$5))^4.5))*Fractions!$B$5*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$F$5&lt;Constants!$B$10,0.002*(E7/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E7/Fractions!$F$5))^4.5))*Fractions!$B$5*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K7">
-        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$E$6&lt;Constants!$B$10,0.002*(E7/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E7/Fractions!$E$6))^4.5))*Fractions!$B$6*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E7&lt;=0,0,IF(E7/Fractions!$F$6&lt;Constants!$B$10,0.002*(E7/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E7/Fractions!$F$6))^4.5))*Fractions!$B$6*F7^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L7">
@@ -3348,23 +3371,23 @@
         <v/>
       </c>
       <c r="G8">
-        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$E$2&lt;Constants!$B$10,0.002*(E8/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E8/Fractions!$E$2))^4.5))*Fractions!$B$2*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$F$2&lt;Constants!$B$10,0.002*(E8/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E8/Fractions!$F$2))^4.5))*Fractions!$B$2*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H8">
-        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$E$3&lt;Constants!$B$10,0.002*(E8/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E8/Fractions!$E$3))^4.5))*Fractions!$B$3*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$F$3&lt;Constants!$B$10,0.002*(E8/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E8/Fractions!$F$3))^4.5))*Fractions!$B$3*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I8">
-        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$E$4&lt;Constants!$B$10,0.002*(E8/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E8/Fractions!$E$4))^4.5))*Fractions!$B$4*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$F$4&lt;Constants!$B$10,0.002*(E8/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E8/Fractions!$F$4))^4.5))*Fractions!$B$4*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J8">
-        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$E$5&lt;Constants!$B$10,0.002*(E8/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E8/Fractions!$E$5))^4.5))*Fractions!$B$5*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$F$5&lt;Constants!$B$10,0.002*(E8/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E8/Fractions!$F$5))^4.5))*Fractions!$B$5*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K8">
-        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$E$6&lt;Constants!$B$10,0.002*(E8/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E8/Fractions!$E$6))^4.5))*Fractions!$B$6*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E8&lt;=0,0,IF(E8/Fractions!$F$6&lt;Constants!$B$10,0.002*(E8/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E8/Fractions!$F$6))^4.5))*Fractions!$B$6*F8^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L8">
@@ -3400,23 +3423,23 @@
         <v/>
       </c>
       <c r="G9">
-        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$E$2&lt;Constants!$B$10,0.002*(E9/Fractions!$E$2)^7.5,14*(1-0.894/SQRT(E9/Fractions!$E$2))^4.5))*Fractions!$B$2*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$F$2&lt;Constants!$B$10,0.002*(E9/Fractions!$F$2)^7.5,14*(1-0.894/SQRT(E9/Fractions!$F$2))^4.5))*Fractions!$B$2*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="H9">
-        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$E$3&lt;Constants!$B$10,0.002*(E9/Fractions!$E$3)^7.5,14*(1-0.894/SQRT(E9/Fractions!$E$3))^4.5))*Fractions!$B$3*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$F$3&lt;Constants!$B$10,0.002*(E9/Fractions!$F$3)^7.5,14*(1-0.894/SQRT(E9/Fractions!$F$3))^4.5))*Fractions!$B$3*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="I9">
-        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$E$4&lt;Constants!$B$10,0.002*(E9/Fractions!$E$4)^7.5,14*(1-0.894/SQRT(E9/Fractions!$E$4))^4.5))*Fractions!$B$4*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$F$4&lt;Constants!$B$10,0.002*(E9/Fractions!$F$4)^7.5,14*(1-0.894/SQRT(E9/Fractions!$F$4))^4.5))*Fractions!$B$4*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="J9">
-        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$E$5&lt;Constants!$B$10,0.002*(E9/Fractions!$E$5)^7.5,14*(1-0.894/SQRT(E9/Fractions!$E$5))^4.5))*Fractions!$B$5*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$F$5&lt;Constants!$B$10,0.002*(E9/Fractions!$F$5)^7.5,14*(1-0.894/SQRT(E9/Fractions!$F$5))^4.5))*Fractions!$B$5*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="K9">
-        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$E$6&lt;Constants!$B$10,0.002*(E9/Fractions!$E$6)^7.5,14*(1-0.894/SQRT(E9/Fractions!$E$6))^4.5))*Fractions!$B$6*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
+        <f>IF(E9&lt;=0,0,IF(E9/Fractions!$F$6&lt;Constants!$B$10,0.002*(E9/Fractions!$F$6)^7.5,14*(1-0.894/SQRT(E9/Fractions!$F$6))^4.5))*Fractions!$B$6*F9^3/((Constants!$B$12-1)*Constants!$B$2)</f>
         <v/>
       </c>
       <c r="L9">

</xml_diff>